<commit_message>
fixed requirements file name
</commit_message>
<xml_diff>
--- a/timesheet_filled.xlsx
+++ b/timesheet_filled.xlsx
@@ -901,7 +901,7 @@
       </c>
       <c r="F3" s="49" t="inlineStr">
         <is>
-          <t>Mar-26</t>
+          <t>Apr-26</t>
         </is>
       </c>
     </row>
@@ -1034,16 +1034,22 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>1 Mar 2026</t>
+          <t>1 Apr 2026</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C10" s="22" t="inlineStr"/>
-      <c r="D10" s="14" t="inlineStr"/>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Development and testing on Co-Delivery project</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E10" s="55" t="n"/>
       <c r="F10" s="51" t="n"/>
       <c r="G10" s="14" t="n"/>
@@ -1051,17 +1057,17 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>2 Mar 2026</t>
+          <t>2 Apr 2026</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C11" s="22" t="inlineStr">
         <is>
-          <t>Development and testing on Co-Delivery project</t>
+          <t>Bug fixing and code review</t>
         </is>
       </c>
       <c r="D11" s="14" t="n">
@@ -1074,17 +1080,17 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>3 Mar 2026</t>
+          <t>3 Apr 2026</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>Bug fixing and code review</t>
+          <t>Feature implementation and documentation</t>
         </is>
       </c>
       <c r="D12" s="14" t="n">
@@ -1097,22 +1103,16 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>4 Mar 2026</t>
+          <t>4 Apr 2026</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="inlineStr">
-        <is>
-          <t>Feature implementation and documentation</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
       <c r="E13" s="55" t="n"/>
       <c r="F13" s="51" t="n"/>
       <c r="G13" s="14" t="n"/>
@@ -1120,22 +1120,16 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>5 Mar 2026</t>
+          <t>5 Apr 2026</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>API development and integration testing</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr"/>
       <c r="E14" s="55" t="n"/>
       <c r="F14" s="51" t="n"/>
       <c r="G14" s="14" t="n"/>
@@ -1143,17 +1137,17 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>6 Mar 2026</t>
+          <t>6 Apr 2026</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Sprint tasks and team collaboration</t>
+          <t>API development and integration testing</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">
@@ -1166,16 +1160,22 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>7 Mar 2026</t>
+          <t>7 Apr 2026</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr"/>
-      <c r="D16" s="14" t="inlineStr"/>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Sprint tasks and team collaboration</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E16" s="56" t="n"/>
       <c r="F16" s="51" t="n"/>
       <c r="G16" s="14" t="n"/>
@@ -1183,16 +1183,22 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>8 Mar 2026</t>
+          <t>8 Apr 2026</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C17" s="24" t="inlineStr"/>
-      <c r="D17" s="23" t="inlineStr"/>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Data pipeline maintenance and monitoring</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="n">
+        <v>1</v>
+      </c>
       <c r="E17" s="57" t="n"/>
       <c r="F17" s="51" t="n"/>
       <c r="G17" s="23" t="n"/>
@@ -1200,17 +1206,17 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>9 Mar 2026</t>
+          <t>9 Apr 2026</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>Data pipeline maintenance and monitoring</t>
+          <t>Database optimization and query tuning</t>
         </is>
       </c>
       <c r="D18" s="23" t="n">
@@ -1229,17 +1235,17 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>10 Mar 2026</t>
+          <t>10 Apr 2026</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>Database optimization and query tuning</t>
+          <t>Unit testing and QA</t>
         </is>
       </c>
       <c r="D19" s="14" t="n">
@@ -1252,22 +1258,16 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>11 Mar 2026</t>
+          <t>11 Apr 2026</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C20" s="22" t="inlineStr">
-        <is>
-          <t>Unit testing and QA</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr"/>
+      <c r="D20" s="14" t="inlineStr"/>
       <c r="E20" s="55" t="n"/>
       <c r="F20" s="51" t="n"/>
       <c r="G20" s="14" t="n"/>
@@ -1275,22 +1275,16 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>12 Mar 2026</t>
+          <t>12 Apr 2026</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>Technical documentation and knowledge sharing</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr"/>
+      <c r="D21" s="14" t="inlineStr"/>
       <c r="E21" s="55" t="n"/>
       <c r="F21" s="51" t="n"/>
       <c r="G21" s="14" t="n"/>
@@ -1298,17 +1292,17 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>13 Mar 2026</t>
+          <t>13 Apr 2026</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Deployment and release management</t>
+          <t>Technical documentation and knowledge sharing</t>
         </is>
       </c>
       <c r="D22" s="14" t="n">
@@ -1321,16 +1315,22 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="13" t="inlineStr">
         <is>
-          <t>14 Mar 2026</t>
+          <t>14 Apr 2026</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr"/>
-      <c r="D23" s="14" t="inlineStr"/>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Deployment and release management</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E23" s="55" t="n"/>
       <c r="F23" s="51" t="n"/>
       <c r="G23" s="14" t="n"/>
@@ -1338,16 +1338,22 @@
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>15 Mar 2026</t>
+          <t>15 Apr 2026</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr"/>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Development and testing on Co-Delivery project</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E24" s="55" t="n"/>
       <c r="F24" s="51" t="n"/>
       <c r="G24" s="14" t="n"/>
@@ -1355,17 +1361,17 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
-          <t>16 Mar 2026</t>
+          <t>16 Apr 2026</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Development and testing on Co-Delivery project</t>
+          <t>Bug fixing and code review</t>
         </is>
       </c>
       <c r="D25" s="14" t="n">
@@ -1378,17 +1384,17 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>17 Mar 2026</t>
+          <t>17 Apr 2026</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Bug fixing and code review</t>
+          <t>Feature implementation and documentation</t>
         </is>
       </c>
       <c r="D26" s="14" t="n">
@@ -1401,22 +1407,16 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>18 Mar 2026</t>
+          <t>18 Apr 2026</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Feature implementation and documentation</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr"/>
       <c r="E27" s="55" t="n"/>
       <c r="F27" s="51" t="n"/>
       <c r="G27" s="14" t="n"/>
@@ -1424,22 +1424,16 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>19 Mar 2026</t>
+          <t>19 Apr 2026</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>API development and integration testing</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr"/>
       <c r="E28" s="55" t="n"/>
       <c r="F28" s="51" t="n"/>
       <c r="G28" s="14" t="n"/>
@@ -1447,17 +1441,17 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>20 Mar 2026</t>
+          <t>20 Apr 2026</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Sprint tasks and team collaboration</t>
+          <t>API development and integration testing</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
@@ -1470,16 +1464,22 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>21 Mar 2026</t>
+          <t>21 Apr 2026</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr"/>
-      <c r="D30" s="14" t="inlineStr"/>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>Sprint tasks and team collaboration</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E30" s="55" t="n"/>
       <c r="F30" s="51" t="n"/>
       <c r="G30" s="14" t="n"/>
@@ -1487,16 +1487,22 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>22 Mar 2026</t>
+          <t>22 Apr 2026</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr"/>
-      <c r="D31" s="14" t="inlineStr"/>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>Data pipeline maintenance and monitoring</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E31" s="55" t="n"/>
       <c r="F31" s="51" t="n"/>
       <c r="G31" s="14" t="n"/>
@@ -1504,17 +1510,17 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>23 Mar 2026</t>
+          <t>23 Apr 2026</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Data pipeline maintenance and monitoring</t>
+          <t>Database optimization and query tuning</t>
         </is>
       </c>
       <c r="D32" s="14" t="n">
@@ -1527,17 +1533,17 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>24 Mar 2026</t>
+          <t>24 Apr 2026</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Fri</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Database optimization and query tuning</t>
+          <t>Unit testing and QA</t>
         </is>
       </c>
       <c r="D33" s="14" t="n">
@@ -1550,22 +1556,16 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>25 Mar 2026</t>
+          <t>25 Apr 2026</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Wed</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>Unit testing and QA</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="14" t="inlineStr"/>
       <c r="E34" s="56" t="n"/>
       <c r="F34" s="51" t="n"/>
       <c r="G34" s="14" t="n"/>
@@ -1573,22 +1573,16 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>26 Mar 2026</t>
+          <t>26 Apr 2026</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Thu</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
-        <is>
-          <t>Technical documentation and knowledge sharing</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="n">
-        <v>1</v>
-      </c>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr"/>
+      <c r="D35" s="14" t="inlineStr"/>
       <c r="E35" s="55" t="n"/>
       <c r="F35" s="51" t="n"/>
       <c r="G35" s="14" t="n"/>
@@ -1596,17 +1590,17 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>27 Mar 2026</t>
+          <t>27 Apr 2026</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>Fri</t>
+          <t>Mon</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Deployment and release management</t>
+          <t>Technical documentation and knowledge sharing</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
@@ -1619,16 +1613,22 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>28 Mar 2026</t>
+          <t>28 Apr 2026</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>Sat</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr"/>
-      <c r="D37" s="14" t="inlineStr"/>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>Deployment and release management</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E37" s="55" t="n"/>
       <c r="F37" s="51" t="n"/>
       <c r="G37" s="14" t="n"/>
@@ -1636,16 +1636,22 @@
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>29 Mar 2026</t>
+          <t>29 Apr 2026</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Sun</t>
-        </is>
-      </c>
-      <c r="C38" s="25" t="inlineStr"/>
-      <c r="D38" s="14" t="inlineStr"/>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C38" s="25" t="inlineStr">
+        <is>
+          <t>Development and testing on Co-Delivery project</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="E38" s="55" t="n"/>
       <c r="F38" s="51" t="n"/>
       <c r="G38" s="14" t="n"/>
@@ -1653,17 +1659,17 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>30 Mar 2026</t>
+          <t>30 Apr 2026</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Mon</t>
+          <t>Thu</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Development and testing on Co-Delivery project</t>
+          <t>Bug fixing and code review</t>
         </is>
       </c>
       <c r="D39" s="14" t="n">
@@ -1674,24 +1680,10 @@
       <c r="G39" s="14" t="n"/>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>31 Mar 2026</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>Tue</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>Bug fixing and code review</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="n">
-        <v>1</v>
-      </c>
+      <c r="A40" s="13" t="inlineStr"/>
+      <c r="B40" s="14" t="inlineStr"/>
+      <c r="C40" s="15" t="inlineStr"/>
+      <c r="D40" s="14" t="inlineStr"/>
       <c r="E40" s="55" t="n"/>
       <c r="F40" s="51" t="n"/>
       <c r="G40" s="14" t="n"/>

</xml_diff>